<commit_message>
Regenerate the published guide at 0.2.0
Rebuilds site/public/ig from the current sources, so the published copy
carries the 0.2.0 version on every artifact and in the package, the
rewritten index page, and the disclaimer that calls the guide a clinical
implementation-support specification.

Built with the terminology server switched off, since tx.fhir.org is not
reachable from this machine: the single validation error and the
warnings all report that codes could not be checked without a
terminology service.

The phrase "decision support" still appears in the generated pages that
render inherited FHIR R4 element definitions, such as the comment on
Patient.gender. That text belongs to the base specification and does not
describe this guide.
</commit_message>
<xml_diff>
--- a/site/public/ig/CodeSystem-heartland-evidence-level.xlsx
+++ b/site/public/ig/CodeSystem-heartland-evidence-level.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-17T14:02:25-04:00</t>
+    <t>2026-09-17T14:11:14-04:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Prepare candidate guide downloads and verify static publication assets
</commit_message>
<xml_diff>
--- a/site/public/ig/CodeSystem-heartland-evidence-level.xlsx
+++ b/site/public/ig/CodeSystem-heartland-evidence-level.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="52">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>0.3.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,19 +48,19 @@
     <t>Status</t>
   </si>
   <si>
-    <t>active</t>
+    <t>draft</t>
   </si>
   <si>
     <t>Experimental</t>
   </si>
   <si>
-    <t>false</t>
+    <t>true</t>
   </si>
   <si>
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-17T14:11:14-04:00</t>
+    <t>2026-09-29T19:00:36-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>Case Sensitive</t>
-  </si>
-  <si>
-    <t>true</t>
   </si>
   <si>
     <t>Value Set (all codes)</t>
@@ -435,53 +432,53 @@
         <v>28</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="B21" t="s" s="2">
         <v>34</v>
-      </c>
-      <c r="B21" t="s" s="2">
-        <v>35</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" s="2"/>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="B23" t="s" s="2">
         <v>37</v>
-      </c>
-      <c r="B23" t="s" s="2">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -496,58 +493,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="B1" t="s" s="1">
         <v>39</v>
       </c>
-      <c r="B1" t="s" s="1">
+      <c r="C1" t="s" s="1">
         <v>40</v>
       </c>
-      <c r="C1" t="s" s="1">
+      <c r="D1" t="s" s="1">
         <v>41</v>
-      </c>
-      <c r="D1" t="s" s="1">
-        <v>42</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="B2" t="s" s="2">
+      <c r="C2" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="C2" t="s" s="2">
+      <c r="D2" t="s" s="2">
         <v>45</v>
-      </c>
-      <c r="D2" t="s" s="2">
-        <v>46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s" s="2">
+        <v>46</v>
+      </c>
+      <c r="C3" t="s" s="2">
         <v>47</v>
       </c>
-      <c r="C3" t="s" s="2">
+      <c r="D3" t="s" s="2">
         <v>48</v>
-      </c>
-      <c r="D3" t="s" s="2">
-        <v>49</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="C4" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="C4" t="s" s="2">
+      <c r="D4" t="s" s="2">
         <v>51</v>
-      </c>
-      <c r="D4" t="s" s="2">
-        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>